<commit_message>
fix(teklif): Vakıfbank IBAN, tam unvan ve vergi bilgisi
- Vakıfbank IBAN'ı şirket tablosundaki doğru numaraya çekildi (…5800 7323…);
  şablonda ilk commit'ten beri …7223… (mod-97 geçersiz) basılıyordu.
  PDF teklif, Sipariş Onay Formu, Excel şablonu ve şablon betiği.
- Tam unvan: Özer Grup Yalıtım İzolasyon A.Ş. (Emrah, 15 Ekim 2026).
- Vergi dairesi Tuzla, VKN 6900279237 (sağlama geçerli); MERSİS boş.
- Tek kalemli teklif tek sayfada kalsın diye hesap sahibi ve vergi satırı
  sıkı düzende yan yana.
- Örnek PDF görseli yeni bilgilerle sitenin kendi PDF yolundan yeniden üretildi.
- tests/pdf/bank-accounts.test.ts: IBAN'lar mod-97 ve tablo kapısı.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/mantolama-teklif-sablonu.xlsx
+++ b/public/templates/mantolama-teklif-sablonu.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
-    <t xml:space="preserve">ÖZERGRUP YALITIM VE İZOLASYON A.Ş.</t>
+    <t xml:space="preserve">ÖZER GRUP YALITIM İZOLASYON A.Ş.</t>
   </si>
   <si>
     <t xml:space="preserve">Mescit Mah. Ulugüney Sk. Harman Plaza A1 Blok K2 No:15 Tuzla / İstanbul</t>
@@ -160,7 +160,7 @@
     <t>VAKIFBANK</t>
   </si>
   <si>
-    <t xml:space="preserve">TR54 0001 5001 5800 7223 2324 14</t>
+    <t xml:space="preserve">TR54 0001 5001 5800 7323 2324 14</t>
   </si>
   <si>
     <t>Nakliye</t>

</xml_diff>